<commit_message>
minor corr 2 disser
</commit_message>
<xml_diff>
--- a/burocracy/svo.xlsx
+++ b/burocracy/svo.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353C1073-966F-4D14-9DEE-538B5BD746AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A09CC4-D04D-45CA-BE27-92B2E6FF0217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0095C8CC-4D13-40B7-BEB9-1D28084485C6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист2" sheetId="2" r:id="rId1"/>
-    <sheet name="Лист1" sheetId="1" r:id="rId2"/>
+    <sheet name="Лист3" sheetId="3" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
+    <sheet name="Лист1" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="list" localSheetId="0">Лист2!$A$1:$B$18</definedName>
+    <definedName name="list" localSheetId="1">Лист2!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
   <si>
     <t>ФИО</t>
   </si>
@@ -190,6 +191,30 @@
   <si>
     <t>Четырехчастотные зеемановские лазерные гироскопы с минимизацией ошибок для высокоточных навигационных систем
 Четырехчастотный лазерный гироскоп зеемановского типа на базе кольцевого гелий-неонового лазера</t>
+  </si>
+  <si>
+    <t>Название</t>
+  </si>
+  <si>
+    <t>Кому писал</t>
+  </si>
+  <si>
+    <t>Статус</t>
+  </si>
+  <si>
+    <t>26/07/31 написал письмо</t>
+  </si>
+  <si>
+    <t>ОИВТ</t>
+  </si>
+  <si>
+    <t>Почта</t>
+  </si>
+  <si>
+    <t>Константин Владимирович Хищенко</t>
+  </si>
+  <si>
+    <t>konst@ihed.ras.ru</t>
   </si>
 </sst>
 </file>
@@ -575,6 +600,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25F923AD-EA8C-4174-ACA4-6D2AC7093DB9}">
+  <dimension ref="B2:E3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" customWidth="1"/>
+    <col min="5" max="5" width="6.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3843722-2CD4-4402-A192-2F9995D934F3}">
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -745,7 +815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD14CDBF-3E99-4578-A70F-AB9B5009F652}">
   <dimension ref="C3:D27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
new diss data add
</commit_message>
<xml_diff>
--- a/burocracy/svo.xlsx
+++ b/burocracy/svo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9B49F6-247D-4784-8798-EBF8B855A92A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027993C7-0F97-4469-AF34-F1E32B79656C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0095C8CC-4D13-40B7-BEB9-1D28084485C6}"/>
   </bookViews>
@@ -227,7 +227,7 @@
     <t>kamch@isan.troitsk.ru</t>
   </si>
   <si>
-    <t>26/08/10 написал письмо</t>
+    <t>Ответил что переслал в ученый совет</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
actual versions folder create
</commit_message>
<xml_diff>
--- a/burocracy/svo.xlsx
+++ b/burocracy/svo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\disser\burocracy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7A7023-074D-435E-82C1-2C88E5381A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC46B09A-3CB7-4C74-B941-06A888B75A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0095C8CC-4D13-40B7-BEB9-1D28084485C6}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="69">
   <si>
     <t>ФИО</t>
   </si>
@@ -254,7 +254,13 @@
     <t>krotov.ua@phystech.edu kryuri@yandex.ru 8-495- 333-00-57</t>
   </si>
   <si>
-    <t>Написал 25/08/26</t>
+    <t>ИРЄ</t>
+  </si>
+  <si>
+    <t>31/08/26 спросил у Лактионова можно ли</t>
+  </si>
+  <si>
+    <t>26/08/31 АВК позвонил Кротову - тот сказал пистаь генеральному. Через форму обратной связи написал - не отправилось, отправил на почту bereg@niipolyus.ru</t>
   </si>
 </sst>
 </file>
@@ -715,7 +721,15 @@
         <v>65</v>
       </c>
       <c r="E5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
         <v>66</v>
+      </c>
+      <c r="E6" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>